<commit_message>
Update mục import số web
</commit_message>
<xml_diff>
--- a/import-so-web.xlsx
+++ b/import-so-web.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
   <si>
     <t>STT</t>
   </si>
@@ -91,6 +91,27 @@
   </si>
   <si>
     <t>đầu</t>
+  </si>
+  <si>
+    <t>Định dạng sim</t>
+  </si>
+  <si>
+    <t>Nhà mạng</t>
+  </si>
+  <si>
+    <t>Gói cước</t>
+  </si>
+  <si>
+    <t>Sim thần tài</t>
+  </si>
+  <si>
+    <t>Viettel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mobifone </t>
+  </si>
+  <si>
+    <t>Sim dễ nhớ</t>
   </si>
 </sst>
 </file>
@@ -409,18 +430,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,34 +457,43 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -475,31 +507,37 @@
         <v>123</v>
       </c>
       <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
         <v>22</v>
       </c>
-      <c r="F2">
+      <c r="I2">
         <v>10000</v>
       </c>
-      <c r="G2">
+      <c r="J2">
         <v>200000</v>
       </c>
-      <c r="H2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2">
+      <c r="K2">
         <v>0</v>
       </c>
-      <c r="J2" t="s">
+      <c r="M2" t="s">
         <v>16</v>
       </c>
-      <c r="K2" t="s">
+      <c r="N2" t="s">
         <v>13</v>
       </c>
-      <c r="L2" t="s">
+      <c r="O2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -513,31 +551,38 @@
         <v>456</v>
       </c>
       <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="F3">
+      <c r="I3">
         <v>50000</v>
       </c>
-      <c r="G3">
+      <c r="J3">
         <v>70000</v>
       </c>
-      <c r="H3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>20</v>
       </c>
-      <c r="J3" t="s">
+      <c r="M3" t="s">
         <v>16</v>
       </c>
-      <c r="K3" t="s">
+      <c r="N3" t="s">
         <v>18</v>
       </c>
-      <c r="L3" t="s">
+      <c r="O3" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>